<commit_message>
July 2026 - working version - core logic changes
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/prototype_untidy.xlsx
+++ b/tests/testthat/testdata/prototype_untidy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rbionline-my.sharepoint.com/personal/igayen_rbi_org_in/Documents/R/Core-Refactor/tidycells/tests/testthat/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="312" documentId="11_EFF234F3807F14A113EB0A40ED825DAB4BC6C160" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A487A923-30EE-4917-9C88-90F33AFBFCBA}"/>
+  <xr:revisionPtr revIDLastSave="330" documentId="11_EFF234F3807F14A113EB0A40ED825DAB4BC6C160" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F93D02CF-7416-4A2B-92B5-5167C319FD13}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Normal" sheetId="2" r:id="rId1"/>
@@ -21,6 +21,26 @@
     <sheet name="Special Case 5" sheetId="8" r:id="rId6"/>
     <sheet name="Sheet - 007" sheetId="1" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="BoxPlot">"BoxPlot"</definedName>
+    <definedName name="Bubble">"Bubble"</definedName>
+    <definedName name="Candlestick">"Candlestick"</definedName>
+    <definedName name="Chart">"Chart"</definedName>
+    <definedName name="ChartImage">"ChartImage"</definedName>
+    <definedName name="ColumnRange">"ColumnRange"</definedName>
+    <definedName name="Dumbbell">"Dumbbell"</definedName>
+    <definedName name="Heatmap">"Heatmap"</definedName>
+    <definedName name="Histogram">"Histogram"</definedName>
+    <definedName name="Map">"Map"</definedName>
+    <definedName name="OHLC">"OHLC"</definedName>
+    <definedName name="PieChart">"PieChart"</definedName>
+    <definedName name="Scatter">"Scatter"</definedName>
+    <definedName name="Series">"Series"</definedName>
+    <definedName name="Stripe">"Stripe"</definedName>
+    <definedName name="Table">"Table"</definedName>
+    <definedName name="TreeMap">"TreeMap"</definedName>
+    <definedName name="Waterfall">"Waterfall"</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
@@ -2093,16 +2113,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2114,14 +2140,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2141,9 +2161,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2181,9 +2201,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2216,9 +2236,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2251,9 +2288,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2461,44 +2515,44 @@
       <c r="C2" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="30" t="s">
         <v>579</v>
       </c>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24" t="s">
+      <c r="E2" s="30"/>
+      <c r="F2" s="30" t="s">
         <v>580</v>
       </c>
-      <c r="G2" s="24"/>
+      <c r="G2" s="30"/>
       <c r="J2" s="2" t="s">
         <v>578</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="30" t="s">
         <v>579</v>
       </c>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24" t="s">
+      <c r="M2" s="30"/>
+      <c r="N2" s="30" t="s">
         <v>580</v>
       </c>
-      <c r="O2" s="24"/>
+      <c r="O2" s="30"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>574</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="25" t="s">
+      <c r="F3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="27" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="2"/>
@@ -2525,10 +2579,10 @@
       <c r="C4" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
       <c r="J4" s="2">
         <v>1</v>
       </c>
@@ -2549,7 +2603,7 @@
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="24" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2585,7 +2639,7 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="23"/>
+      <c r="B6" s="24"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
@@ -2601,7 +2655,7 @@
       <c r="G6" s="1">
         <v>5416</v>
       </c>
-      <c r="J6" s="23" t="s">
+      <c r="J6" s="24" t="s">
         <v>5</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -2617,7 +2671,7 @@
       <c r="O6" s="15"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="23"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
@@ -2633,7 +2687,7 @@
       <c r="G7" s="1">
         <v>10283</v>
       </c>
-      <c r="J7" s="23"/>
+      <c r="J7" s="24"/>
       <c r="K7" s="2" t="s">
         <v>12</v>
       </c>
@@ -2649,7 +2703,7 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B8" s="23"/>
+      <c r="B8" s="24"/>
       <c r="C8" s="2" t="s">
         <v>36</v>
       </c>
@@ -2663,7 +2717,7 @@
       <c r="G8" s="1">
         <v>9446</v>
       </c>
-      <c r="J8" s="23"/>
+      <c r="J8" s="24"/>
       <c r="K8" s="2" t="s">
         <v>23</v>
       </c>
@@ -2679,7 +2733,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="24" t="s">
         <v>48</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -2697,7 +2751,7 @@
       <c r="G9" s="1">
         <v>10166</v>
       </c>
-      <c r="J9" s="23"/>
+      <c r="J9" s="24"/>
       <c r="K9" s="2" t="s">
         <v>36</v>
       </c>
@@ -2711,7 +2765,7 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="23"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="2" t="s">
         <v>12</v>
       </c>
@@ -2727,7 +2781,7 @@
       <c r="G10" s="1">
         <v>7782</v>
       </c>
-      <c r="J10" s="23" t="s">
+      <c r="J10" s="24" t="s">
         <v>48</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -2745,7 +2799,7 @@
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="23"/>
+      <c r="B11" s="24"/>
       <c r="C11" s="2" t="s">
         <v>23</v>
       </c>
@@ -2761,7 +2815,7 @@
       <c r="G11" s="1">
         <v>7100</v>
       </c>
-      <c r="J11" s="23"/>
+      <c r="J11" s="24"/>
       <c r="K11" s="2" t="s">
         <v>12</v>
       </c>
@@ -2777,7 +2831,7 @@
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="23"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="2" t="s">
         <v>36</v>
       </c>
@@ -2793,7 +2847,7 @@
       <c r="G12" s="1">
         <v>8719</v>
       </c>
-      <c r="J12" s="23"/>
+      <c r="J12" s="24"/>
       <c r="K12" s="2" t="s">
         <v>23</v>
       </c>
@@ -2809,7 +2863,7 @@
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="24" t="s">
         <v>94</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -2825,7 +2879,7 @@
       <c r="G13" s="1">
         <v>9413</v>
       </c>
-      <c r="J13" s="23"/>
+      <c r="J13" s="24"/>
       <c r="K13" s="2" t="s">
         <v>36</v>
       </c>
@@ -2841,7 +2895,7 @@
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="23"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="2" t="s">
         <v>12</v>
       </c>
@@ -2857,7 +2911,7 @@
       <c r="G14" s="1">
         <v>8823</v>
       </c>
-      <c r="J14" s="23" t="s">
+      <c r="J14" s="24" t="s">
         <v>94</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -2876,7 +2930,7 @@
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="23"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2892,7 +2946,7 @@
       <c r="G15" s="1">
         <v>8913</v>
       </c>
-      <c r="J15" s="23"/>
+      <c r="J15" s="24"/>
       <c r="K15" s="2" t="s">
         <v>12</v>
       </c>
@@ -2908,7 +2962,7 @@
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="23"/>
+      <c r="B16" s="24"/>
       <c r="C16" s="2" t="s">
         <v>36</v>
       </c>
@@ -2924,7 +2978,7 @@
       <c r="G16" s="1">
         <v>9340</v>
       </c>
-      <c r="J16" s="23"/>
+      <c r="J16" s="24"/>
       <c r="K16" s="2" t="s">
         <v>23</v>
       </c>
@@ -2940,7 +2994,7 @@
       </c>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="24" t="s">
         <v>140</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -2958,7 +3012,7 @@
       <c r="G17" s="1">
         <v>6006</v>
       </c>
-      <c r="J17" s="23"/>
+      <c r="J17" s="24"/>
       <c r="K17" s="2" t="s">
         <v>36</v>
       </c>
@@ -2974,7 +3028,7 @@
       </c>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B18" s="23"/>
+      <c r="B18" s="24"/>
       <c r="C18" s="2" t="s">
         <v>12</v>
       </c>
@@ -2990,7 +3044,7 @@
       <c r="G18" s="1">
         <v>13652</v>
       </c>
-      <c r="J18" s="23" t="s">
+      <c r="J18" s="24" t="s">
         <v>140</v>
       </c>
       <c r="K18" s="2" t="s">
@@ -3008,7 +3062,7 @@
       </c>
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B19" s="23"/>
+      <c r="B19" s="24"/>
       <c r="C19" s="2" t="s">
         <v>23</v>
       </c>
@@ -3024,7 +3078,7 @@
       <c r="G19" s="1">
         <v>11188</v>
       </c>
-      <c r="J19" s="23"/>
+      <c r="J19" s="24"/>
       <c r="K19" s="2" t="s">
         <v>12</v>
       </c>
@@ -3040,7 +3094,7 @@
       </c>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="23"/>
+      <c r="B20" s="24"/>
       <c r="C20" s="2" t="s">
         <v>36</v>
       </c>
@@ -3056,7 +3110,7 @@
       <c r="G20" s="1">
         <v>12909</v>
       </c>
-      <c r="J20" s="23"/>
+      <c r="J20" s="24"/>
       <c r="K20" s="2" t="s">
         <v>23</v>
       </c>
@@ -3072,7 +3126,7 @@
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="24" t="s">
         <v>188</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -3082,7 +3136,7 @@
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
-      <c r="J21" s="23"/>
+      <c r="J21" s="24"/>
       <c r="K21" s="2" t="s">
         <v>36</v>
       </c>
@@ -3098,7 +3152,7 @@
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" s="23"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="2" t="s">
         <v>12</v>
       </c>
@@ -3114,7 +3168,7 @@
       <c r="G22" s="1">
         <v>10300</v>
       </c>
-      <c r="J22" s="23" t="s">
+      <c r="J22" s="24" t="s">
         <v>188</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -3128,7 +3182,7 @@
       <c r="O22" s="15"/>
     </row>
     <row r="23" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B23" s="23"/>
+      <c r="B23" s="24"/>
       <c r="C23" s="2" t="s">
         <v>23</v>
       </c>
@@ -3144,7 +3198,7 @@
       <c r="G23" s="1">
         <v>8754</v>
       </c>
-      <c r="J23" s="23"/>
+      <c r="J23" s="24"/>
       <c r="K23" s="2" t="s">
         <v>12</v>
       </c>
@@ -3162,7 +3216,7 @@
       </c>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B24" s="23"/>
+      <c r="B24" s="24"/>
       <c r="C24" s="2" t="s">
         <v>36</v>
       </c>
@@ -3174,7 +3228,7 @@
       <c r="G24" s="1">
         <v>15786</v>
       </c>
-      <c r="J24" s="23"/>
+      <c r="J24" s="24"/>
       <c r="K24" s="2" t="s">
         <v>23</v>
       </c>
@@ -3192,7 +3246,7 @@
       </c>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="J25" s="23"/>
+      <c r="J25" s="24"/>
       <c r="K25" s="2" t="s">
         <v>36</v>
       </c>
@@ -3220,7 +3274,7 @@
       <c r="F30" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G30" s="23" t="s">
+      <c r="G30" s="24" t="s">
         <v>5</v>
       </c>
       <c r="J30" s="10"/>
@@ -3232,7 +3286,7 @@
       <c r="N30" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O30" s="28" t="s">
+      <c r="O30" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -3246,7 +3300,7 @@
       <c r="F31" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G31" s="23"/>
+      <c r="G31" s="24"/>
       <c r="J31" s="10"/>
       <c r="K31" s="10"/>
       <c r="L31" s="10"/>
@@ -3256,7 +3310,7 @@
       <c r="N31" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O31" s="29"/>
+      <c r="O31" s="22"/>
     </row>
     <row r="32" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B32" s="10"/>
@@ -3268,7 +3322,7 @@
       <c r="F32" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G32" s="23"/>
+      <c r="G32" s="24"/>
       <c r="J32" s="10"/>
       <c r="K32" s="10"/>
       <c r="L32" s="10"/>
@@ -3278,7 +3332,7 @@
       <c r="N32" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O32" s="29"/>
+      <c r="O32" s="22"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B33" s="10"/>
@@ -3290,7 +3344,7 @@
       <c r="F33" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G33" s="23"/>
+      <c r="G33" s="24"/>
       <c r="J33" s="10"/>
       <c r="K33" s="10"/>
       <c r="L33" s="10"/>
@@ -3300,7 +3354,7 @@
       <c r="N33" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="O33" s="30"/>
+      <c r="O33" s="23"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B34" s="10"/>
@@ -3312,7 +3366,7 @@
       <c r="F34" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G34" s="23" t="s">
+      <c r="G34" s="24" t="s">
         <v>48</v>
       </c>
       <c r="J34" s="10"/>
@@ -3324,7 +3378,7 @@
       <c r="N34" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O34" s="28" t="s">
+      <c r="O34" s="21" t="s">
         <v>48</v>
       </c>
     </row>
@@ -3342,7 +3396,7 @@
       <c r="F35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="23"/>
+      <c r="G35" s="24"/>
       <c r="J35" s="1">
         <v>9892</v>
       </c>
@@ -3356,7 +3410,7 @@
       <c r="N35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O35" s="29"/>
+      <c r="O35" s="22"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B36" s="1">
@@ -3372,7 +3426,7 @@
       <c r="F36" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G36" s="23"/>
+      <c r="G36" s="24"/>
       <c r="J36" s="1">
         <v>8623</v>
       </c>
@@ -3386,7 +3440,7 @@
       <c r="N36" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O36" s="29"/>
+      <c r="O36" s="22"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B37" s="1">
@@ -3402,7 +3456,7 @@
       <c r="F37" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G37" s="23"/>
+      <c r="G37" s="24"/>
       <c r="J37" s="1">
         <v>5775</v>
       </c>
@@ -3416,7 +3470,7 @@
       <c r="N37" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="O37" s="30"/>
+      <c r="O37" s="23"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
@@ -3430,7 +3484,7 @@
       <c r="F38" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G38" s="23" t="s">
+      <c r="G38" s="24" t="s">
         <v>94</v>
       </c>
       <c r="J38" s="1"/>
@@ -3444,7 +3498,7 @@
       <c r="N38" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O38" s="28" t="s">
+      <c r="O38" s="21" t="s">
         <v>94</v>
       </c>
     </row>
@@ -3462,7 +3516,7 @@
       <c r="F39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G39" s="23"/>
+      <c r="G39" s="24"/>
       <c r="J39" s="1">
         <v>8770</v>
       </c>
@@ -3476,7 +3530,7 @@
       <c r="N39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O39" s="29"/>
+      <c r="O39" s="22"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B40" s="1">
@@ -3492,7 +3546,7 @@
       <c r="F40" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G40" s="23"/>
+      <c r="G40" s="24"/>
       <c r="J40" s="1">
         <v>7389</v>
       </c>
@@ -3506,7 +3560,7 @@
       <c r="N40" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O40" s="29"/>
+      <c r="O40" s="22"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
@@ -3525,7 +3579,7 @@
       <c r="F41" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G41" s="23"/>
+      <c r="G41" s="24"/>
       <c r="J41" s="1">
         <v>15204</v>
       </c>
@@ -3539,7 +3593,7 @@
       <c r="N41" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="O41" s="30"/>
+      <c r="O41" s="23"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B42" s="1">
@@ -3555,7 +3609,7 @@
       <c r="F42" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G42" s="23" t="s">
+      <c r="G42" s="24" t="s">
         <v>140</v>
       </c>
       <c r="J42" s="1">
@@ -3571,7 +3625,7 @@
       <c r="N42" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O42" s="28" t="s">
+      <c r="O42" s="21" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3589,7 +3643,7 @@
       <c r="F43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G43" s="23"/>
+      <c r="G43" s="24"/>
       <c r="J43" s="1">
         <v>16109</v>
       </c>
@@ -3603,7 +3657,7 @@
       <c r="N43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O43" s="29"/>
+      <c r="O43" s="22"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B44" s="1">
@@ -3619,7 +3673,7 @@
       <c r="F44" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G44" s="23"/>
+      <c r="G44" s="24"/>
       <c r="J44" s="1">
         <v>12640</v>
       </c>
@@ -3633,7 +3687,7 @@
       <c r="N44" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O44" s="29"/>
+      <c r="O44" s="22"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B45" s="1">
@@ -3649,7 +3703,7 @@
       <c r="F45" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G45" s="23"/>
+      <c r="G45" s="24"/>
       <c r="J45" s="1">
         <v>9020</v>
       </c>
@@ -3663,7 +3717,7 @@
       <c r="N45" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="O45" s="30"/>
+      <c r="O45" s="23"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B46" s="10"/>
@@ -3673,7 +3727,7 @@
       <c r="F46" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G46" s="23" t="s">
+      <c r="G46" s="24" t="s">
         <v>188</v>
       </c>
       <c r="J46" s="10"/>
@@ -3683,7 +3737,7 @@
       <c r="N46" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O46" s="28" t="s">
+      <c r="O46" s="21" t="s">
         <v>188</v>
       </c>
     </row>
@@ -3703,7 +3757,7 @@
       <c r="F47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G47" s="23"/>
+      <c r="G47" s="24"/>
       <c r="J47" s="1">
         <v>10480</v>
       </c>
@@ -3719,7 +3773,7 @@
       <c r="N47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O47" s="29"/>
+      <c r="O47" s="22"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B48" s="1">
@@ -3737,7 +3791,7 @@
       <c r="F48" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G48" s="23"/>
+      <c r="G48" s="24"/>
       <c r="J48" s="1">
         <v>10200</v>
       </c>
@@ -3753,7 +3807,7 @@
       <c r="N48" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O48" s="29"/>
+      <c r="O48" s="22"/>
     </row>
     <row r="49" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
@@ -3767,7 +3821,7 @@
       <c r="F49" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G49" s="23"/>
+      <c r="G49" s="24"/>
       <c r="J49" s="1"/>
       <c r="K49" s="1">
         <v>8795</v>
@@ -3779,7 +3833,7 @@
       <c r="N49" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="O49" s="30"/>
+      <c r="O49" s="23"/>
     </row>
     <row r="50" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B50" s="13" t="s">
@@ -3854,14 +3908,14 @@
       </c>
     </row>
     <row r="52" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B52" s="24" t="s">
+      <c r="B52" s="30" t="s">
         <v>579</v>
       </c>
-      <c r="C52" s="24"/>
-      <c r="D52" s="24" t="s">
+      <c r="C52" s="30"/>
+      <c r="D52" s="30" t="s">
         <v>580</v>
       </c>
-      <c r="E52" s="24"/>
+      <c r="E52" s="30"/>
       <c r="F52" s="2" t="s">
         <v>577</v>
       </c>
@@ -3898,10 +3952,10 @@
       <c r="P53" s="20">
         <v>0</v>
       </c>
-      <c r="R53" s="27" t="s">
+      <c r="R53" s="29" t="s">
         <v>586</v>
       </c>
-      <c r="S53" s="27"/>
+      <c r="S53" s="29"/>
     </row>
     <row r="54" spans="2:19" x14ac:dyDescent="0.25">
       <c r="J54" s="20">
@@ -3927,7 +3981,7 @@
       </c>
     </row>
     <row r="56" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B56" s="23" t="s">
+      <c r="B56" s="24" t="s">
         <v>5</v>
       </c>
       <c r="C56" s="2" t="s">
@@ -3943,7 +3997,7 @@
       <c r="G56" s="15"/>
     </row>
     <row r="57" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B57" s="23"/>
+      <c r="B57" s="24"/>
       <c r="C57" s="2" t="s">
         <v>12</v>
       </c>
@@ -3959,7 +4013,7 @@
       </c>
     </row>
     <row r="58" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="23"/>
+      <c r="B58" s="24"/>
       <c r="C58" s="2" t="s">
         <v>23</v>
       </c>
@@ -3975,7 +4029,7 @@
       </c>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B59" s="23"/>
+      <c r="B59" s="24"/>
       <c r="C59" s="2" t="s">
         <v>36</v>
       </c>
@@ -3993,17 +4047,17 @@
       <c r="L59" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="M59" s="21" t="s">
+      <c r="M59" s="25" t="s">
         <v>579</v>
       </c>
-      <c r="N59" s="22"/>
-      <c r="P59" s="21" t="s">
+      <c r="N59" s="26"/>
+      <c r="P59" s="25" t="s">
         <v>580</v>
       </c>
-      <c r="Q59" s="22"/>
+      <c r="Q59" s="26"/>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B60" s="23" t="s">
+      <c r="B60" s="24" t="s">
         <v>48</v>
       </c>
       <c r="C60" s="2" t="s">
@@ -4021,21 +4075,21 @@
       <c r="L60" s="2" t="s">
         <v>574</v>
       </c>
-      <c r="M60" s="25" t="s">
+      <c r="M60" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="N60" s="25" t="s">
+      <c r="N60" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="P60" s="25" t="s">
+      <c r="P60" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="Q60" s="25" t="s">
+      <c r="Q60" s="27" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="61" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="23"/>
+      <c r="B61" s="24"/>
       <c r="C61" s="2" t="s">
         <v>12</v>
       </c>
@@ -4053,13 +4107,13 @@
       <c r="L61" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="M61" s="26"/>
-      <c r="N61" s="26"/>
-      <c r="P61" s="26"/>
-      <c r="Q61" s="26"/>
+      <c r="M61" s="28"/>
+      <c r="N61" s="28"/>
+      <c r="P61" s="28"/>
+      <c r="Q61" s="28"/>
     </row>
     <row r="62" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B62" s="23"/>
+      <c r="B62" s="24"/>
       <c r="C62" s="2" t="s">
         <v>23</v>
       </c>
@@ -4071,7 +4125,7 @@
       </c>
       <c r="F62" s="15"/>
       <c r="G62" s="15"/>
-      <c r="K62" s="28" t="s">
+      <c r="K62" s="21" t="s">
         <v>5</v>
       </c>
       <c r="L62" s="2" t="s">
@@ -4089,7 +4143,7 @@
       </c>
     </row>
     <row r="63" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="23"/>
+      <c r="B63" s="24"/>
       <c r="C63" s="2" t="s">
         <v>36</v>
       </c>
@@ -4101,7 +4155,7 @@
       </c>
       <c r="F63" s="15"/>
       <c r="G63" s="15"/>
-      <c r="K63" s="29"/>
+      <c r="K63" s="22"/>
       <c r="L63" s="2" t="s">
         <v>12</v>
       </c>
@@ -4119,7 +4173,7 @@
       </c>
     </row>
     <row r="64" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="23" t="s">
+      <c r="B64" s="24" t="s">
         <v>94</v>
       </c>
       <c r="C64" s="2" t="s">
@@ -4134,7 +4188,7 @@
       <c r="I64" s="11" t="s">
         <v>584</v>
       </c>
-      <c r="K64" s="29"/>
+      <c r="K64" s="22"/>
       <c r="L64" s="2" t="s">
         <v>23</v>
       </c>
@@ -4152,7 +4206,7 @@
       </c>
     </row>
     <row r="65" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B65" s="23"/>
+      <c r="B65" s="24"/>
       <c r="C65" s="2" t="s">
         <v>12</v>
       </c>
@@ -4164,7 +4218,7 @@
       </c>
       <c r="F65" s="15"/>
       <c r="G65" s="15"/>
-      <c r="K65" s="30"/>
+      <c r="K65" s="23"/>
       <c r="L65" s="2" t="s">
         <v>36</v>
       </c>
@@ -4180,7 +4234,7 @@
       </c>
     </row>
     <row r="66" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B66" s="23"/>
+      <c r="B66" s="24"/>
       <c r="C66" s="2" t="s">
         <v>23</v>
       </c>
@@ -4194,7 +4248,7 @@
       <c r="G66" s="15"/>
     </row>
     <row r="67" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B67" s="23"/>
+      <c r="B67" s="24"/>
       <c r="C67" s="2" t="s">
         <v>36</v>
       </c>
@@ -4206,7 +4260,7 @@
       </c>
       <c r="F67" s="15"/>
       <c r="G67" s="15"/>
-      <c r="K67" s="28" t="s">
+      <c r="K67" s="21" t="s">
         <v>48</v>
       </c>
       <c r="L67" s="2" t="s">
@@ -4226,7 +4280,7 @@
       </c>
     </row>
     <row r="68" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B68" s="23" t="s">
+      <c r="B68" s="24" t="s">
         <v>140</v>
       </c>
       <c r="C68" s="2" t="s">
@@ -4240,7 +4294,7 @@
       </c>
       <c r="F68" s="15"/>
       <c r="G68" s="15"/>
-      <c r="K68" s="29"/>
+      <c r="K68" s="22"/>
       <c r="L68" s="2" t="s">
         <v>12</v>
       </c>
@@ -4258,7 +4312,7 @@
       </c>
     </row>
     <row r="69" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B69" s="23"/>
+      <c r="B69" s="24"/>
       <c r="C69" s="2" t="s">
         <v>12</v>
       </c>
@@ -4270,7 +4324,7 @@
       </c>
       <c r="F69" s="15"/>
       <c r="G69" s="15"/>
-      <c r="K69" s="29"/>
+      <c r="K69" s="22"/>
       <c r="L69" s="2" t="s">
         <v>23</v>
       </c>
@@ -4288,7 +4342,7 @@
       </c>
     </row>
     <row r="70" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B70" s="23"/>
+      <c r="B70" s="24"/>
       <c r="C70" s="2" t="s">
         <v>23</v>
       </c>
@@ -4300,7 +4354,7 @@
       </c>
       <c r="F70" s="15"/>
       <c r="G70" s="15"/>
-      <c r="K70" s="30"/>
+      <c r="K70" s="23"/>
       <c r="L70" s="2" t="s">
         <v>36</v>
       </c>
@@ -4318,7 +4372,7 @@
       </c>
     </row>
     <row r="71" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B71" s="23"/>
+      <c r="B71" s="24"/>
       <c r="C71" s="2" t="s">
         <v>36</v>
       </c>
@@ -4332,7 +4386,7 @@
       <c r="G71" s="15"/>
     </row>
     <row r="72" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B72" s="23" t="s">
+      <c r="B72" s="24" t="s">
         <v>188</v>
       </c>
       <c r="C72" s="2" t="s">
@@ -4344,7 +4398,7 @@
       </c>
       <c r="F72" s="15"/>
       <c r="G72" s="15"/>
-      <c r="K72" s="28" t="s">
+      <c r="K72" s="21" t="s">
         <v>94</v>
       </c>
       <c r="L72" s="2" t="s">
@@ -4362,7 +4416,7 @@
       </c>
     </row>
     <row r="73" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B73" s="23"/>
+      <c r="B73" s="24"/>
       <c r="C73" s="2" t="s">
         <v>12</v>
       </c>
@@ -4378,7 +4432,7 @@
       <c r="G73" s="1">
         <v>10300</v>
       </c>
-      <c r="K73" s="29"/>
+      <c r="K73" s="22"/>
       <c r="L73" s="2" t="s">
         <v>12</v>
       </c>
@@ -4396,7 +4450,7 @@
       </c>
     </row>
     <row r="74" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B74" s="23"/>
+      <c r="B74" s="24"/>
       <c r="C74" s="2" t="s">
         <v>23</v>
       </c>
@@ -4412,7 +4466,7 @@
       <c r="G74" s="1">
         <v>8754</v>
       </c>
-      <c r="K74" s="29"/>
+      <c r="K74" s="22"/>
       <c r="L74" s="2" t="s">
         <v>23</v>
       </c>
@@ -4430,7 +4484,7 @@
       </c>
     </row>
     <row r="75" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B75" s="23"/>
+      <c r="B75" s="24"/>
       <c r="C75" s="2" t="s">
         <v>36</v>
       </c>
@@ -4442,7 +4496,7 @@
       <c r="G75" s="1">
         <v>15786</v>
       </c>
-      <c r="K75" s="30"/>
+      <c r="K75" s="23"/>
       <c r="L75" s="2" t="s">
         <v>36</v>
       </c>
@@ -4474,15 +4528,15 @@
       </c>
     </row>
     <row r="77" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="D77" s="24" t="s">
+      <c r="D77" s="30" t="s">
         <v>579</v>
       </c>
-      <c r="E77" s="24"/>
-      <c r="F77" s="21" t="s">
+      <c r="E77" s="30"/>
+      <c r="F77" s="25" t="s">
         <v>580</v>
       </c>
-      <c r="G77" s="22"/>
-      <c r="K77" s="28" t="s">
+      <c r="G77" s="26"/>
+      <c r="K77" s="21" t="s">
         <v>140</v>
       </c>
       <c r="L77" s="2" t="s">
@@ -4502,7 +4556,7 @@
       </c>
     </row>
     <row r="78" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K78" s="29"/>
+      <c r="K78" s="22"/>
       <c r="L78" s="2" t="s">
         <v>12</v>
       </c>
@@ -4520,7 +4574,7 @@
       </c>
     </row>
     <row r="79" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K79" s="29"/>
+      <c r="K79" s="22"/>
       <c r="L79" s="2" t="s">
         <v>23</v>
       </c>
@@ -4538,7 +4592,7 @@
       </c>
     </row>
     <row r="80" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K80" s="30"/>
+      <c r="K80" s="23"/>
       <c r="L80" s="2" t="s">
         <v>36</v>
       </c>
@@ -4561,7 +4615,7 @@
       </c>
     </row>
     <row r="82" spans="11:19" x14ac:dyDescent="0.25">
-      <c r="K82" s="23" t="s">
+      <c r="K82" s="24" t="s">
         <v>188</v>
       </c>
       <c r="L82" s="2" t="s">
@@ -4573,7 +4627,7 @@
       <c r="Q82" s="10"/>
     </row>
     <row r="83" spans="11:19" x14ac:dyDescent="0.25">
-      <c r="K83" s="23"/>
+      <c r="K83" s="24"/>
       <c r="L83" s="2" t="s">
         <v>12</v>
       </c>
@@ -4591,7 +4645,7 @@
       </c>
     </row>
     <row r="84" spans="11:19" x14ac:dyDescent="0.25">
-      <c r="K84" s="23"/>
+      <c r="K84" s="24"/>
       <c r="L84" s="2" t="s">
         <v>23</v>
       </c>
@@ -4609,7 +4663,7 @@
       </c>
     </row>
     <row r="85" spans="11:19" x14ac:dyDescent="0.25">
-      <c r="K85" s="23"/>
+      <c r="K85" s="24"/>
       <c r="L85" s="2" t="s">
         <v>36</v>
       </c>
@@ -4624,28 +4678,18 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="O42:O45"/>
-    <mergeCell ref="K62:K65"/>
-    <mergeCell ref="K67:K70"/>
-    <mergeCell ref="K72:K75"/>
-    <mergeCell ref="K77:K80"/>
-    <mergeCell ref="K82:K85"/>
-    <mergeCell ref="M59:N59"/>
-    <mergeCell ref="M60:M61"/>
-    <mergeCell ref="N60:N61"/>
-    <mergeCell ref="R53:S53"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="J22:J25"/>
-    <mergeCell ref="J18:J21"/>
-    <mergeCell ref="O38:O41"/>
-    <mergeCell ref="O34:O37"/>
-    <mergeCell ref="O30:O33"/>
-    <mergeCell ref="Q60:Q61"/>
-    <mergeCell ref="P60:P61"/>
-    <mergeCell ref="P59:Q59"/>
-    <mergeCell ref="O46:O49"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="B72:B75"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="B60:B63"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="J6:J9"/>
+    <mergeCell ref="J10:J13"/>
+    <mergeCell ref="J14:J17"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="B5:B8"/>
@@ -4655,24 +4699,34 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="G3:G4"/>
+    <mergeCell ref="O38:O41"/>
+    <mergeCell ref="O34:O37"/>
+    <mergeCell ref="O30:O33"/>
+    <mergeCell ref="Q60:Q61"/>
+    <mergeCell ref="P60:P61"/>
+    <mergeCell ref="P59:Q59"/>
+    <mergeCell ref="O46:O49"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="J22:J25"/>
+    <mergeCell ref="J18:J21"/>
     <mergeCell ref="B17:B20"/>
     <mergeCell ref="G38:G41"/>
     <mergeCell ref="G42:G45"/>
     <mergeCell ref="G46:G49"/>
     <mergeCell ref="G30:G33"/>
     <mergeCell ref="G34:G37"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="J6:J9"/>
-    <mergeCell ref="J10:J13"/>
-    <mergeCell ref="J14:J17"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="B72:B75"/>
-    <mergeCell ref="D77:E77"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="K82:K85"/>
+    <mergeCell ref="M59:N59"/>
+    <mergeCell ref="M60:M61"/>
+    <mergeCell ref="N60:N61"/>
+    <mergeCell ref="R53:S53"/>
+    <mergeCell ref="O42:O45"/>
+    <mergeCell ref="K62:K65"/>
+    <mergeCell ref="K67:K70"/>
+    <mergeCell ref="K72:K75"/>
+    <mergeCell ref="K77:K80"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4685,7 +4739,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -4703,7 +4757,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="23"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4721,7 +4775,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
+      <c r="A4" s="24"/>
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
@@ -4739,7 +4793,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="23"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="2" t="s">
         <v>36</v>
       </c>
@@ -4755,7 +4809,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="24" t="s">
         <v>48</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -4775,7 +4829,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
@@ -4793,7 +4847,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="23"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="2" t="s">
         <v>23</v>
       </c>
@@ -4811,7 +4865,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="23"/>
+      <c r="A9" s="24"/>
       <c r="B9" s="2" t="s">
         <v>36</v>
       </c>
@@ -4829,7 +4883,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="24" t="s">
         <v>94</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -4847,7 +4901,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="23"/>
+      <c r="A11" s="24"/>
       <c r="B11" s="2" t="s">
         <v>12</v>
       </c>
@@ -4865,7 +4919,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
+      <c r="A12" s="24"/>
       <c r="B12" s="2" t="s">
         <v>23</v>
       </c>
@@ -4883,7 +4937,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="2" t="s">
         <v>36</v>
       </c>
@@ -4901,7 +4955,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="24" t="s">
         <v>140</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -4921,7 +4975,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="23"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="2" t="s">
         <v>12</v>
       </c>
@@ -4939,7 +4993,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="23"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="2" t="s">
         <v>23</v>
       </c>
@@ -4957,7 +5011,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="23"/>
+      <c r="A17" s="24"/>
       <c r="B17" s="2" t="s">
         <v>36</v>
       </c>
@@ -4975,7 +5029,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="24" t="s">
         <v>188</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -4987,7 +5041,7 @@
       <c r="F18" s="10"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="23"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="2" t="s">
         <v>12</v>
       </c>
@@ -5005,7 +5059,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="23"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="2" t="s">
         <v>23</v>
       </c>
@@ -5023,7 +5077,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="23"/>
+      <c r="A21" s="24"/>
       <c r="B21" s="2" t="s">
         <v>36</v>
       </c>
@@ -5064,7 +5118,7 @@
       <c r="F7" s="1">
         <v>13394</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="24" t="s">
         <v>5</v>
       </c>
     </row>
@@ -5075,7 +5129,7 @@
       <c r="F8" s="1">
         <v>5416</v>
       </c>
-      <c r="G8" s="23"/>
+      <c r="G8" s="24"/>
     </row>
     <row r="9" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C9" s="10"/>
@@ -5084,7 +5138,7 @@
       <c r="F9" s="1">
         <v>10283</v>
       </c>
-      <c r="G9" s="23"/>
+      <c r="G9" s="24"/>
     </row>
     <row r="10" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C10" s="10"/>
@@ -5093,7 +5147,7 @@
       <c r="F10" s="1">
         <v>9446</v>
       </c>
-      <c r="G10" s="23"/>
+      <c r="G10" s="24"/>
     </row>
     <row r="11" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C11" s="10"/>
@@ -5102,7 +5156,7 @@
       <c r="F11" s="1">
         <v>10166</v>
       </c>
-      <c r="G11" s="23"/>
+      <c r="G11" s="24"/>
     </row>
     <row r="12" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C12" s="1">
@@ -5115,7 +5169,7 @@
       <c r="F12" s="1">
         <v>7782</v>
       </c>
-      <c r="G12" s="23"/>
+      <c r="G12" s="24"/>
     </row>
     <row r="13" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C13" s="1">
@@ -5128,7 +5182,7 @@
       <c r="F13" s="1">
         <v>7100</v>
       </c>
-      <c r="G13" s="23"/>
+      <c r="G13" s="24"/>
     </row>
     <row r="14" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C14" s="1">
@@ -5141,7 +5195,7 @@
       <c r="F14" s="1">
         <v>8719</v>
       </c>
-      <c r="G14" s="23"/>
+      <c r="G14" s="24"/>
     </row>
     <row r="15" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C15" s="1"/>
@@ -5152,7 +5206,7 @@
       <c r="F15" s="1">
         <v>9413</v>
       </c>
-      <c r="G15" s="23"/>
+      <c r="G15" s="24"/>
     </row>
     <row r="16" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C16" s="1">
@@ -5165,7 +5219,7 @@
       <c r="F16" s="1">
         <v>8823</v>
       </c>
-      <c r="G16" s="23"/>
+      <c r="G16" s="24"/>
     </row>
     <row r="17" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C17" s="1">
@@ -5178,7 +5232,7 @@
       <c r="F17" s="1">
         <v>8913</v>
       </c>
-      <c r="G17" s="23"/>
+      <c r="G17" s="24"/>
     </row>
     <row r="18" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C18" s="1">
@@ -5191,7 +5245,7 @@
       <c r="F18" s="1">
         <v>9340</v>
       </c>
-      <c r="G18" s="23"/>
+      <c r="G18" s="24"/>
     </row>
     <row r="19" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C19" s="1">
@@ -5204,7 +5258,7 @@
       <c r="F19" s="1">
         <v>6006</v>
       </c>
-      <c r="G19" s="23"/>
+      <c r="G19" s="24"/>
     </row>
     <row r="20" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C20" s="1">
@@ -5217,7 +5271,7 @@
       <c r="F20" s="1">
         <v>13652</v>
       </c>
-      <c r="G20" s="23"/>
+      <c r="G20" s="24"/>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C21" s="1">
@@ -5230,7 +5284,7 @@
       <c r="F21" s="1">
         <v>11188</v>
       </c>
-      <c r="G21" s="23"/>
+      <c r="G21" s="24"/>
     </row>
     <row r="22" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C22" s="1">
@@ -5243,14 +5297,14 @@
       <c r="F22" s="1">
         <v>12909</v>
       </c>
-      <c r="G22" s="23"/>
+      <c r="G22" s="24"/>
     </row>
     <row r="23" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="1"/>
-      <c r="G23" s="23"/>
+      <c r="G23" s="24"/>
     </row>
     <row r="24" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C24" s="1">
@@ -5265,7 +5319,7 @@
       <c r="F24" s="1">
         <v>10300</v>
       </c>
-      <c r="G24" s="23"/>
+      <c r="G24" s="24"/>
     </row>
     <row r="25" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C25" s="1">
@@ -5280,7 +5334,7 @@
       <c r="F25" s="1">
         <v>8754</v>
       </c>
-      <c r="G25" s="23"/>
+      <c r="G25" s="24"/>
     </row>
     <row r="26" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C26" s="1"/>
@@ -5291,7 +5345,7 @@
       <c r="F26" s="1">
         <v>15786</v>
       </c>
-      <c r="G26" s="23"/>
+      <c r="G26" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -6060,14 +6114,14 @@
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24" t="s">
+      <c r="E2" s="30"/>
+      <c r="F2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="24"/>
+      <c r="G2" s="30"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="D3" s="2" t="s">
@@ -6084,7 +6138,7 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -6108,7 +6162,7 @@
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B5" s="23"/>
+      <c r="B5" s="24"/>
       <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
@@ -6152,7 +6206,7 @@
       <c r="Y5" s="2"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B6" s="23"/>
+      <c r="B6" s="24"/>
       <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6201,7 +6255,7 @@
       <c r="Y6" s="2"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B7" s="23"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="2" t="s">
         <v>36</v>
       </c>
@@ -6248,7 +6302,7 @@
       <c r="Y7" s="2"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="24" t="s">
         <v>48</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -6299,7 +6353,7 @@
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B9" s="23"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="2" t="s">
         <v>12</v>
       </c>
@@ -6348,7 +6402,7 @@
       <c r="Y9" s="2"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B10" s="23"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
@@ -6397,7 +6451,7 @@
       <c r="Y10" s="2"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B11" s="23"/>
+      <c r="B11" s="24"/>
       <c r="C11" s="2" t="s">
         <v>36</v>
       </c>
@@ -6446,7 +6500,7 @@
       <c r="Y11" s="2"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="24" t="s">
         <v>94</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -6500,7 +6554,7 @@
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B13" s="23"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="2" t="s">
         <v>12</v>
       </c>
@@ -6544,7 +6598,7 @@
       <c r="Y13" s="2"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B14" s="23"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="2" t="s">
         <v>23</v>
       </c>
@@ -6593,7 +6647,7 @@
       <c r="Y14" s="2"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B15" s="23"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="2" t="s">
         <v>36</v>
       </c>
@@ -6642,7 +6696,7 @@
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="24" t="s">
         <v>140</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -6698,7 +6752,7 @@
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B17" s="23"/>
+      <c r="B17" s="24"/>
       <c r="C17" s="2" t="s">
         <v>12</v>
       </c>
@@ -6747,7 +6801,7 @@
       <c r="Y17" s="2"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B18" s="23"/>
+      <c r="B18" s="24"/>
       <c r="C18" s="2" t="s">
         <v>23</v>
       </c>
@@ -6796,7 +6850,7 @@
       <c r="Y18" s="2"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B19" s="23"/>
+      <c r="B19" s="24"/>
       <c r="C19" s="2" t="s">
         <v>36</v>
       </c>
@@ -6845,7 +6899,7 @@
       <c r="Y19" s="2"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="24" t="s">
         <v>188</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -6895,7 +6949,7 @@
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B21" s="23"/>
+      <c r="B21" s="24"/>
       <c r="C21" s="2" t="s">
         <v>12</v>
       </c>
@@ -6927,7 +6981,7 @@
       <c r="Y21" s="2"/>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B22" s="23"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="2" t="s">
         <v>23</v>
       </c>
@@ -6976,7 +7030,7 @@
       <c r="Y22" s="2"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B23" s="23"/>
+      <c r="B23" s="24"/>
       <c r="C23" s="2" t="s">
         <v>36</v>
       </c>

</xml_diff>